<commit_message>
Major update. Questions 1-20 completed. 5 to go. Will. My. Sanity. Last?
</commit_message>
<xml_diff>
--- a/Status Tracker.xlsx
+++ b/Status Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bradspoerri/DS5010/project_jpy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB23CAB-21E4-4B42-8BC2-58BA28D69D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844D5944-1F74-0A4B-BDE4-A6A81EBCBC1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19420" xr2:uid="{16D847D7-7B4E-C14C-8F49-633BE51E8839}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19480" xr2:uid="{16D847D7-7B4E-C14C-8F49-633BE51E8839}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Status</t>
   </si>
@@ -53,120 +53,83 @@
     <t>Exciting Insights (any technique)</t>
   </si>
   <si>
-    <t>Distribution of combined dataset by type (does this align with regional production?)</t>
-  </si>
-  <si>
-    <t>Create a function to classify wines as "Dry," "Off-Dry," "Semi-Sweet," or "Sweet" based on residual sugar levels. How much do wines with similar or the same physiochemical properties differ?</t>
-  </si>
-  <si>
-    <t>How does sulphate content vary by type of wine?</t>
-  </si>
-  <si>
-    <t>Use a lambda function to categorize alcohol content into "Low" (&lt;10%), "Medium" (10-12%), and "High" (&gt;12%). What's the distribution across quality ratings?</t>
-  </si>
-  <si>
-    <t>Write a function that calculates the "acidity ratio" (fixed acidity / volatile acidity)</t>
-  </si>
-  <si>
-    <t>Which physicochemical properties are most closely related? (correlation)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Distribution of quality scores by type </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(average quality and sd by type)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve"> What physiochemical properties have the most significant impact on overall quality?</t>
-  </si>
-  <si>
-    <t>Write function to find chemical outliers (explore if this impacts quality)</t>
-  </si>
-  <si>
-    <t>What is the average rating per type of wine?</t>
-  </si>
-  <si>
-    <t>What is the range in quality for each type of wine?</t>
-  </si>
-  <si>
-    <r>
-      <t>What is the average alcohol content for each quality rating?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Does higher alcohol correlate with higher quality?</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Which physicochemical property has the highest variance</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> across all wines? Does this differ between red and white?</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Group wines by quality and calculate the mean of all physicochemical properties.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Which properties change most dramatically across quality levels?</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Create a heatmap of the correlation matrix.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Which features are most/least correlated with quality?</t>
-    </r>
-  </si>
-  <si>
-    <t>ANOVA on quality by type</t>
-  </si>
-  <si>
-    <t>Does the data follow a normal distribution?</t>
-  </si>
-  <si>
-    <t>Which properties have the greatest range per quality rating and type?</t>
+    <t>Create a function to classify wines as "Dry," "Off-Dry," "Semi-Sweet," or "Sweet" based on residual sugar levels.</t>
+  </si>
+  <si>
+    <t>Create a bar chart of quality ratings after grouping the data by type?</t>
+  </si>
+  <si>
+    <t>How does sweetness vary between the different types of wine?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the distribution of quality scores by type of wine? </t>
+  </si>
+  <si>
+    <t>Which features are most/least correlated with quality?</t>
+  </si>
+  <si>
+    <t>Create a heatmap of the correlation matrix.</t>
+  </si>
+  <si>
+    <t>How do chemical markers differ between wine types?</t>
+  </si>
+  <si>
+    <t>Box plots</t>
+  </si>
+  <si>
+    <t>How does the ratio of fixed to volatile differ by type of wine?</t>
+  </si>
+  <si>
+    <t>Distribution of acidity ratio by wine type (hist)</t>
+  </si>
+  <si>
+    <t>How does free sulfur (sulfite) content compare by wine type and does it have any clear impact on quality rating?</t>
+  </si>
+  <si>
+    <t>Histogram of distribution + line graph with sd error bars</t>
+  </si>
+  <si>
+    <t>Does acohol have a clear impact on quality?</t>
+  </si>
+  <si>
+    <t>Plot mean alcohol by quality with std error bar</t>
+  </si>
+  <si>
+    <t>Do any outlier groupings appear to have a significant impact on quality?</t>
+  </si>
+  <si>
+    <t>Data frames by type of wine and type of outlier</t>
+  </si>
+  <si>
+    <t>How many outliers are there for each chemical marker (3xMAD from Mean)?</t>
+  </si>
+  <si>
+    <t>Do sulphates impact the ratio of free sulfur to total sulfur?</t>
+  </si>
+  <si>
+    <t>Scatter plot and line plot with std error bars</t>
+  </si>
+  <si>
+    <t>How do alcohol content and wine density relate to one another?</t>
+  </si>
+  <si>
+    <t>Box plot of densities for each abv bin (5 bins)</t>
+  </si>
+  <si>
+    <t>Function to calculate MAD then prepare df with count of 3MAD outliers</t>
+  </si>
+  <si>
+    <t>What percentage of each type of wine is premium? (quality &gt; 7)</t>
+  </si>
+  <si>
+    <t>agg lambda function</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -184,12 +147,6 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -227,7 +184,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -413,23 +370,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -441,7 +431,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -466,7 +456,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -479,14 +469,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -822,254 +826,298 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A8597EC-0A79-3E46-ABE8-5106E60D5F5D}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="58" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="7.1640625" style="1"/>
+    <col min="2" max="2" width="51.1640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="58" style="1" customWidth="1"/>
+    <col min="4" max="6" width="7.1640625" style="1"/>
+    <col min="7" max="7" width="49.1640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="7.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="11">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="6"/>
-    </row>
-    <row r="3" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="B2" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="18"/>
+    </row>
+    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="13">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="7"/>
-    </row>
-    <row r="4" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B3" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="19"/>
+    </row>
+    <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="13">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="7"/>
-    </row>
-    <row r="5" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="19"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="13">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="7"/>
-    </row>
-    <row r="6" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="32"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16">
         <v>5</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="8"/>
-    </row>
-    <row r="7" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="30"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="21"/>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B7" s="31"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="11">
         <v>1</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="18"/>
-    </row>
-    <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B8" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="18"/>
+    </row>
+    <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
         <v>2</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="19"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B9" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="19"/>
+    </row>
+    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="13">
         <v>3</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B10" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="19"/>
+    </row>
+    <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="13">
         <v>4</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="7"/>
-    </row>
-    <row r="12" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B11" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="19"/>
+    </row>
+    <row r="12" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="13">
         <v>5</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="7"/>
-    </row>
-    <row r="13" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B12" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="19"/>
+    </row>
+    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="13">
         <v>6</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="7"/>
-    </row>
-    <row r="14" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B13" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="19"/>
+    </row>
+    <row r="14" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="13">
         <v>7</v>
       </c>
-      <c r="B14" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="7"/>
-    </row>
-    <row r="15" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="B14" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="19"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="13">
         <v>8</v>
       </c>
-      <c r="B15" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="19"/>
-    </row>
-    <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B15" s="32"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="33"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="13">
         <v>9</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="32"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="7"/>
+    </row>
+    <row r="17" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="16">
         <v>10</v>
       </c>
-      <c r="B17" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="8"/>
-    </row>
-    <row r="18" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="35"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="8"/>
+    </row>
+    <row r="18" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B18" s="31"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="11">
         <v>1</v>
       </c>
-      <c r="B19" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B19" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="18"/>
+    </row>
+    <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="13">
         <v>2</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="7"/>
-    </row>
-    <row r="21" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B20" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="19"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="13">
         <v>3</v>
       </c>
-      <c r="B21" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="7"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B21" s="29"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="7"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="13">
         <v>4</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="7"/>
-    </row>
-    <row r="23" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="29"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="7"/>
+    </row>
+    <row r="23" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="16">
         <v>5</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="8"/>
-    </row>
-    <row r="24" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="30"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="8"/>
+    </row>
+    <row r="24" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="5"/>
-    </row>
-    <row r="25" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B24" s="31"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="5"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="11">
         <v>1</v>
       </c>
-      <c r="B25" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="6"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B25" s="28"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="6"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="13">
         <v>2</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="7"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B26" s="29"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="7"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="13">
         <v>3</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="7"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B27" s="29"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="13">
         <v>4</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="7"/>
-    </row>
-    <row r="29" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="29"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="7"/>
+    </row>
+    <row r="29" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16">
         <v>5</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="8"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>